<commit_message>
Modified the Dashboard image
</commit_message>
<xml_diff>
--- a/analysis/UK_Inflation_Analysis.xlsx
+++ b/analysis/UK_Inflation_Analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Poorva JV\Documents\GitHub\UK-Inflation-Tracker\analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA7CAFC7-ED35-428E-9B10-2428C89D23E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DDC516B-7F7F-4CAC-9141-FE354F6B7C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{F829807F-E675-4258-B921-BB8B5220F5FE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{F829807F-E675-4258-B921-BB8B5220F5FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="2" r:id="rId1"/>
@@ -76,9 +76,6 @@
     <t>Change in Inflation rate (pp)</t>
   </si>
   <si>
-    <t>The largest annual increase in the inflation rate within this period occurred in 2022.</t>
-  </si>
-  <si>
     <t>UK Inflation Dashboard</t>
   </si>
   <si>
@@ -124,10 +121,13 @@
     <t>Insights:</t>
   </si>
   <si>
-    <t>Inflation subsequently declined</t>
+    <t>Inflation peaked at 9.1% in 2022, representing the highest rate in the period analysed.</t>
   </si>
   <si>
-    <t>The inflation rate decreased by 6.6 percentage points.</t>
+    <t>Following the 2022 peak, inflation declined to 7.3% in 2023 and 2.5% in 2024.</t>
+  </si>
+  <si>
+    <t>Inflation declined by 6.6 percentage points between 2022 and 2024.</t>
   </si>
 </sst>
 </file>
@@ -137,7 +137,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -300,14 +300,6 @@
     </font>
     <font>
       <b/>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="16"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -315,7 +307,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Display"/>
@@ -510,7 +501,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="25">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -635,10 +626,109 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top style="thin">
-        <color theme="5"/>
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -648,131 +738,7 @@
       <right/>
       <top/>
       <bottom style="thin">
-        <color theme="5"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color theme="1" tint="4.9989318521683403E-2"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color theme="1" tint="4.9989318521683403E-2"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color theme="1" tint="4.9989318521683403E-2"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color theme="1" tint="4.9989318521683403E-2"/>
-      </right>
-      <top style="medium">
-        <color theme="1" tint="4.9989318521683403E-2"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color theme="1" tint="4.9989318521683403E-2"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color theme="1" tint="4.9989318521683403E-2"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color theme="1" tint="4.9989318521683403E-2"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color theme="5"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color theme="1" tint="4.9989318521683403E-2"/>
-      </right>
-      <top style="thin">
-        <color theme="5"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color theme="1" tint="4.9989318521683403E-2"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color theme="5"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color theme="1" tint="4.9989318521683403E-2"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color theme="5"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color theme="1" tint="4.9989318521683403E-2"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="1" tint="4.9989318521683403E-2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="1" tint="4.9989318521683403E-2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color theme="1" tint="4.9989318521683403E-2"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color theme="1" tint="4.9989318521683403E-2"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -821,67 +787,86 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="18" fillId="33" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="22" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1011,7 +996,17 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.11197667320696292"/>
+          <c:y val="0.12458130054668462"/>
+          <c:w val="0.84839211409060455"/>
+          <c:h val="0.71088534090191546"/>
+        </c:manualLayout>
+      </c:layout>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
@@ -1177,7 +1172,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1050" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1100" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:ln>
                       <a:noFill/>
                     </a:ln>
@@ -1190,7 +1185,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-IN" sz="1050"/>
+                  <a:rPr lang="en-IN" sz="1100"/>
                   <a:t>Year</a:t>
                 </a:r>
               </a:p>
@@ -1209,7 +1204,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1050" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1100" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:ln>
                     <a:noFill/>
                   </a:ln>
@@ -1247,7 +1242,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:ln>
                   <a:noFill/>
                 </a:ln>
@@ -1294,7 +1289,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1050" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1150" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:ln>
                       <a:noFill/>
                     </a:ln>
@@ -1307,7 +1302,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-IN" sz="1050"/>
+                  <a:rPr lang="en-IN" sz="1150"/>
                   <a:t>Inflation rate (%)</a:t>
                 </a:r>
               </a:p>
@@ -1326,7 +1321,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1050" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1150" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:ln>
                     <a:noFill/>
                   </a:ln>
@@ -1994,13 +1989,13 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>27878</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>49250</xdr:rowOff>
+      <xdr:colOff>167268</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>148683</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>594731</xdr:colOff>
+      <xdr:colOff>548268</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>176561</xdr:rowOff>
     </xdr:to>
@@ -2484,32 +2479,32 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -2585,7 +2580,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C9">
         <f>MEDIAN(Data!B2:B11)</f>
@@ -2594,7 +2589,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C10">
         <f>DEVSQ(Data!B2:B11)</f>
@@ -2603,7 +2598,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C11">
         <f>MAX(Data!C3:C11)</f>
@@ -2612,7 +2607,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C12">
         <f>MIN(Data!C3:C11)</f>
@@ -2635,267 +2630,505 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11670F5B-AA1D-4803-9D80-46DAAEBFEC46}">
-  <dimension ref="B1:K33"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="2:11" s="7" customFormat="1" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C1" s="6"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
-    </row>
-    <row r="2" spans="2:11" s="7" customFormat="1" ht="15" x14ac:dyDescent="0.35">
-      <c r="B2" s="19"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-      <c r="J2" s="20"/>
-      <c r="K2" s="22"/>
-    </row>
-    <row r="3" spans="2:11" ht="27" x14ac:dyDescent="0.6">
-      <c r="B3" s="23"/>
-      <c r="D3" s="34" t="s">
+    <row r="1" spans="1:12" s="4" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+      <c r="C1" s="3"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+    </row>
+    <row r="2" spans="1:12" s="4" customFormat="1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A2" s="34"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="36"/>
+      <c r="I2" s="36"/>
+      <c r="J2" s="35"/>
+      <c r="K2" s="35"/>
+      <c r="L2" s="37"/>
+    </row>
+    <row r="3" spans="1:12" ht="27" x14ac:dyDescent="0.6">
+      <c r="A3" s="38"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
+      <c r="L3" s="39"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" s="38"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
+      <c r="L4" s="39"/>
+    </row>
+    <row r="5" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="38"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="24"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="34"/>
-      <c r="H3" s="34"/>
-      <c r="I3" s="34"/>
-      <c r="K3" s="24"/>
-    </row>
-    <row r="4" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B4" s="23"/>
-      <c r="K4" s="24"/>
-    </row>
-    <row r="5" spans="2:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="23"/>
-      <c r="C5" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="11"/>
-      <c r="F5" s="35" t="s">
+      <c r="G5" s="20"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="G5" s="35"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="35" t="s">
-        <v>16</v>
-      </c>
-      <c r="J5" s="35"/>
-      <c r="K5" s="24"/>
-    </row>
-    <row r="6" spans="2:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="23"/>
-      <c r="C6" s="13">
+      <c r="J5" s="20"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="39"/>
+    </row>
+    <row r="6" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="38"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="15">
         <f>Analysis!C4</f>
         <v>3.01</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="D6" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="F6" s="13">
+      <c r="E6" s="6"/>
+      <c r="F6" s="15">
         <f>Analysis!C5</f>
         <v>9.1</v>
       </c>
-      <c r="G6" s="12" t="s">
+      <c r="G6" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="H6" s="3"/>
-      <c r="I6" s="13">
+      <c r="H6" s="8"/>
+      <c r="I6" s="15">
         <f>Analysis!C6</f>
         <v>0.7</v>
       </c>
-      <c r="J6" s="12" t="s">
+      <c r="J6" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="K6" s="24"/>
-    </row>
-    <row r="7" spans="2:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="23"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="10"/>
-      <c r="K7" s="24"/>
-    </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B8" s="23"/>
-      <c r="K8" s="24"/>
-    </row>
-    <row r="9" spans="2:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="23"/>
-      <c r="K9" s="24"/>
-    </row>
-    <row r="10" spans="2:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="23"/>
-      <c r="K10" s="24"/>
-    </row>
-    <row r="11" spans="2:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="23"/>
-      <c r="K11" s="24"/>
-    </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B12" s="23"/>
-      <c r="K12" s="24"/>
-    </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B13" s="23"/>
-      <c r="K13" s="24"/>
-    </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B14" s="23"/>
-      <c r="K14" s="24"/>
-    </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B15" s="23"/>
-      <c r="K15" s="24"/>
-    </row>
-    <row r="16" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B16" s="23"/>
-      <c r="K16" s="24"/>
-    </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B17" s="23"/>
-      <c r="K17" s="24"/>
-    </row>
-    <row r="18" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B18" s="23"/>
-      <c r="K18" s="24"/>
-    </row>
-    <row r="19" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B19" s="23"/>
-      <c r="K19" s="24"/>
-    </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B20" s="23"/>
-      <c r="K20" s="24"/>
-    </row>
-    <row r="21" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B21" s="23"/>
-      <c r="K21" s="24"/>
-    </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B22" s="23"/>
-      <c r="K22" s="24"/>
-    </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B23" s="23"/>
-      <c r="K23" s="24"/>
-    </row>
-    <row r="24" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B24" s="23"/>
-      <c r="K24" s="24"/>
-    </row>
-    <row r="25" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B25" s="23"/>
-      <c r="K25" s="24"/>
-    </row>
-    <row r="26" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B26" s="23"/>
-      <c r="K26" s="24"/>
-    </row>
-    <row r="27" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B27" s="23"/>
-      <c r="K27" s="24"/>
-    </row>
-    <row r="28" spans="2:11" ht="21" x14ac:dyDescent="0.3">
+      <c r="K6" s="6"/>
+      <c r="L6" s="39"/>
+    </row>
+    <row r="7" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="38"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="39"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8" s="38"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="6"/>
+      <c r="K8" s="6"/>
+      <c r="L8" s="39"/>
+    </row>
+    <row r="9" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="38"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="6"/>
+      <c r="K9" s="6"/>
+      <c r="L9" s="39"/>
+    </row>
+    <row r="10" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="38"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="6"/>
+      <c r="K10" s="6"/>
+      <c r="L10" s="39"/>
+    </row>
+    <row r="11" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="38"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6"/>
+      <c r="L11" s="39"/>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A12" s="38"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="6"/>
+      <c r="K12" s="6"/>
+      <c r="L12" s="39"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A13" s="38"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6"/>
+      <c r="L13" s="39"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A14" s="38"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="6"/>
+      <c r="K14" s="6"/>
+      <c r="L14" s="39"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A15" s="38"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6"/>
+      <c r="I15" s="6"/>
+      <c r="J15" s="6"/>
+      <c r="K15" s="6"/>
+      <c r="L15" s="39"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A16" s="38"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+      <c r="I16" s="6"/>
+      <c r="J16" s="6"/>
+      <c r="K16" s="6"/>
+      <c r="L16" s="39"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A17" s="38"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="6"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="6"/>
+      <c r="K17" s="6"/>
+      <c r="L17" s="39"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A18" s="38"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6"/>
+      <c r="H18" s="6"/>
+      <c r="I18" s="6"/>
+      <c r="J18" s="6"/>
+      <c r="K18" s="6"/>
+      <c r="L18" s="39"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A19" s="38"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="6"/>
+      <c r="K19" s="6"/>
+      <c r="L19" s="39"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A20" s="38"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+      <c r="I20" s="6"/>
+      <c r="J20" s="6"/>
+      <c r="K20" s="6"/>
+      <c r="L20" s="39"/>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A21" s="38"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="6"/>
+      <c r="K21" s="6"/>
+      <c r="L21" s="39"/>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A22" s="38"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="6"/>
+      <c r="H22" s="6"/>
+      <c r="I22" s="6"/>
+      <c r="J22" s="6"/>
+      <c r="K22" s="6"/>
+      <c r="L22" s="39"/>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A23" s="38"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="6"/>
+      <c r="K23" s="6"/>
+      <c r="L23" s="39"/>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A24" s="38"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+      <c r="I24" s="6"/>
+      <c r="J24" s="6"/>
+      <c r="K24" s="6"/>
+      <c r="L24" s="39"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A25" s="38"/>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="6"/>
+      <c r="H25" s="6"/>
+      <c r="I25" s="6"/>
+      <c r="J25" s="6"/>
+      <c r="K25" s="6"/>
+      <c r="L25" s="39"/>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A26" s="38"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
+      <c r="I26" s="6"/>
+      <c r="J26" s="6"/>
+      <c r="K26" s="6"/>
+      <c r="L26" s="39"/>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A27" s="38"/>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+      <c r="I27" s="6"/>
+      <c r="J27" s="6"/>
+      <c r="K27" s="6"/>
+      <c r="L27" s="39"/>
+    </row>
+    <row r="28" spans="1:12" ht="21" x14ac:dyDescent="0.3">
+      <c r="A28" s="38"/>
       <c r="B28" s="25"/>
-      <c r="C28" s="14" t="s">
+      <c r="C28" s="26" t="s">
+        <v>27</v>
+      </c>
+      <c r="D28" s="27"/>
+      <c r="E28" s="27"/>
+      <c r="F28" s="27"/>
+      <c r="G28" s="27"/>
+      <c r="H28" s="27"/>
+      <c r="I28" s="27"/>
+      <c r="J28" s="27"/>
+      <c r="K28" s="28"/>
+      <c r="L28" s="39"/>
+    </row>
+    <row r="29" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A29" s="38"/>
+      <c r="B29" s="29"/>
+      <c r="C29" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="D28" s="15"/>
-      <c r="E28" s="15"/>
-      <c r="F28" s="15"/>
-      <c r="G28" s="15"/>
-      <c r="H28" s="15"/>
-      <c r="I28" s="15"/>
-      <c r="J28" s="15"/>
-      <c r="K28" s="26"/>
-    </row>
-    <row r="29" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B29" s="27"/>
-      <c r="C29" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="D29" s="17"/>
-      <c r="E29" s="17"/>
-      <c r="F29" s="17"/>
-      <c r="G29" s="17"/>
-      <c r="H29" s="17"/>
-      <c r="I29" s="17"/>
-      <c r="J29" s="17"/>
-      <c r="K29" s="28"/>
-    </row>
-    <row r="30" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B30" s="27"/>
-      <c r="C30" s="16" t="s">
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="30"/>
+      <c r="L29" s="39"/>
+    </row>
+    <row r="30" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A30" s="38"/>
+      <c r="B30" s="29"/>
+      <c r="C30" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="D30" s="17"/>
-      <c r="E30" s="17"/>
-      <c r="F30" s="17"/>
-      <c r="G30" s="17"/>
-      <c r="H30" s="17"/>
-      <c r="I30" s="17"/>
-      <c r="J30" s="17"/>
-      <c r="K30" s="28"/>
-    </row>
-    <row r="31" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B31" s="27"/>
-      <c r="C31" s="16" t="s">
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="10"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="10"/>
+      <c r="J30" s="10"/>
+      <c r="K30" s="30"/>
+      <c r="L30" s="39"/>
+    </row>
+    <row r="31" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A31" s="38"/>
+      <c r="B31" s="29"/>
+      <c r="C31" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
-      <c r="F31" s="17"/>
-      <c r="G31" s="17"/>
-      <c r="H31" s="17"/>
-      <c r="I31" s="17"/>
-      <c r="J31" s="17"/>
-      <c r="K31" s="28"/>
-    </row>
-    <row r="32" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B32" s="29"/>
-      <c r="C32" s="18"/>
-      <c r="D32" s="18"/>
-      <c r="E32" s="18"/>
-      <c r="F32" s="18"/>
-      <c r="G32" s="18"/>
-      <c r="H32" s="18"/>
-      <c r="I32" s="18"/>
-      <c r="J32" s="18"/>
-      <c r="K32" s="30"/>
-    </row>
-    <row r="33" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="31"/>
-      <c r="C33" s="32"/>
-      <c r="D33" s="32"/>
-      <c r="E33" s="32"/>
-      <c r="F33" s="32"/>
-      <c r="G33" s="32"/>
-      <c r="H33" s="32"/>
-      <c r="I33" s="32"/>
-      <c r="J33" s="32"/>
-      <c r="K33" s="33"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="10"/>
+      <c r="H31" s="10"/>
+      <c r="I31" s="10"/>
+      <c r="J31" s="10"/>
+      <c r="K31" s="30"/>
+      <c r="L31" s="39"/>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A32" s="38"/>
+      <c r="B32" s="31"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="32"/>
+      <c r="G32" s="32"/>
+      <c r="H32" s="32"/>
+      <c r="I32" s="32"/>
+      <c r="J32" s="32"/>
+      <c r="K32" s="33"/>
+      <c r="L32" s="39"/>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A33" s="40"/>
+      <c r="B33" s="41"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="41"/>
+      <c r="G33" s="41"/>
+      <c r="H33" s="41"/>
+      <c r="I33" s="41"/>
+      <c r="J33" s="41"/>
+      <c r="K33" s="41"/>
+      <c r="L33" s="42"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="D3:I3"/>
     <mergeCell ref="I5:J5"/>
     <mergeCell ref="F5:G5"/>
+    <mergeCell ref="C5:D5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>